<commit_message>
Refresh button in student results
</commit_message>
<xml_diff>
--- a/publish/questions.xlsx
+++ b/publish/questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\anuj\opnsrc_try\ai\QuizWeb_Manual\publish\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7ADB591-00DF-4CE2-9C77-F0260C063358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F988492E-D102-419F-98D8-43D4626BD81A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="679">
   <si>
     <t>Class: 9</t>
   </si>
@@ -2057,12 +2057,6 @@
   </si>
   <si>
     <t>Numbers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? What does HTML stand for? </t>
-  </si>
-  <si>
-    <t>images/triangle.png</t>
   </si>
 </sst>
 </file>
@@ -2966,14 +2960,8 @@
       <c r="A5" t="s">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
-        <v>679</v>
-      </c>
       <c r="C5" t="s">
         <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>680</v>
       </c>
       <c r="E5" t="s">
         <v>19</v>
@@ -2998,14 +2986,8 @@
       <c r="A6" t="s">
         <v>25</v>
       </c>
-      <c r="B6" t="s">
-        <v>679</v>
-      </c>
       <c r="C6" t="s">
         <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>680</v>
       </c>
       <c r="E6" t="s">
         <v>27</v>
@@ -3030,14 +3012,8 @@
       <c r="A7" t="s">
         <v>33</v>
       </c>
-      <c r="B7" t="s">
-        <v>679</v>
-      </c>
       <c r="C7" t="s">
         <v>34</v>
-      </c>
-      <c r="D7" t="s">
-        <v>680</v>
       </c>
       <c r="E7" t="s">
         <v>35</v>
@@ -3062,14 +3038,8 @@
       <c r="A8" t="s">
         <v>41</v>
       </c>
-      <c r="B8" t="s">
-        <v>679</v>
-      </c>
       <c r="C8" t="s">
         <v>42</v>
-      </c>
-      <c r="D8" t="s">
-        <v>680</v>
       </c>
       <c r="E8" t="s">
         <v>43</v>
@@ -3094,14 +3064,8 @@
       <c r="A9" t="s">
         <v>49</v>
       </c>
-      <c r="B9" t="s">
-        <v>679</v>
-      </c>
       <c r="C9" t="s">
         <v>50</v>
-      </c>
-      <c r="D9" t="s">
-        <v>680</v>
       </c>
       <c r="E9" t="s">
         <v>51</v>
@@ -3126,14 +3090,8 @@
       <c r="A10" t="s">
         <v>57</v>
       </c>
-      <c r="B10" t="s">
-        <v>679</v>
-      </c>
       <c r="C10" t="s">
         <v>58</v>
-      </c>
-      <c r="D10" t="s">
-        <v>680</v>
       </c>
       <c r="E10" t="s">
         <v>19</v>
@@ -3158,14 +3116,8 @@
       <c r="A11" t="s">
         <v>64</v>
       </c>
-      <c r="B11" t="s">
-        <v>679</v>
-      </c>
       <c r="C11" t="s">
         <v>65</v>
-      </c>
-      <c r="D11" t="s">
-        <v>680</v>
       </c>
       <c r="E11" t="s">
         <v>27</v>
@@ -3190,14 +3142,8 @@
       <c r="A12" t="s">
         <v>71</v>
       </c>
-      <c r="B12" t="s">
-        <v>679</v>
-      </c>
       <c r="C12" t="s">
         <v>72</v>
-      </c>
-      <c r="D12" t="s">
-        <v>680</v>
       </c>
       <c r="E12" t="s">
         <v>35</v>
@@ -3222,14 +3168,8 @@
       <c r="A13" t="s">
         <v>74</v>
       </c>
-      <c r="B13" t="s">
-        <v>679</v>
-      </c>
       <c r="C13" t="s">
         <v>75</v>
-      </c>
-      <c r="D13" t="s">
-        <v>680</v>
       </c>
       <c r="E13" t="s">
         <v>43</v>
@@ -3254,14 +3194,8 @@
       <c r="A14" t="s">
         <v>78</v>
       </c>
-      <c r="B14" t="s">
-        <v>679</v>
-      </c>
       <c r="C14" t="s">
         <v>79</v>
-      </c>
-      <c r="D14" t="s">
-        <v>680</v>
       </c>
       <c r="E14" t="s">
         <v>51</v>
@@ -3286,14 +3220,8 @@
       <c r="A15" t="s">
         <v>85</v>
       </c>
-      <c r="B15" t="s">
-        <v>679</v>
-      </c>
       <c r="C15" t="s">
         <v>86</v>
-      </c>
-      <c r="D15" t="s">
-        <v>680</v>
       </c>
       <c r="E15" t="s">
         <v>19</v>
@@ -3318,14 +3246,8 @@
       <c r="A16" t="s">
         <v>88</v>
       </c>
-      <c r="B16" t="s">
-        <v>679</v>
-      </c>
       <c r="C16" t="s">
         <v>89</v>
-      </c>
-      <c r="D16" t="s">
-        <v>680</v>
       </c>
       <c r="E16" t="s">
         <v>27</v>
@@ -3350,14 +3272,8 @@
       <c r="A17" t="s">
         <v>92</v>
       </c>
-      <c r="B17" t="s">
-        <v>679</v>
-      </c>
       <c r="C17" t="s">
         <v>93</v>
-      </c>
-      <c r="D17" t="s">
-        <v>680</v>
       </c>
       <c r="E17" t="s">
         <v>35</v>
@@ -3382,14 +3298,8 @@
       <c r="A18" t="s">
         <v>95</v>
       </c>
-      <c r="B18" t="s">
-        <v>679</v>
-      </c>
       <c r="C18" t="s">
         <v>96</v>
-      </c>
-      <c r="D18" t="s">
-        <v>680</v>
       </c>
       <c r="E18" t="s">
         <v>43</v>
@@ -3414,14 +3324,8 @@
       <c r="A19" t="s">
         <v>102</v>
       </c>
-      <c r="B19" t="s">
-        <v>679</v>
-      </c>
       <c r="C19" t="s">
         <v>103</v>
-      </c>
-      <c r="D19" t="s">
-        <v>680</v>
       </c>
       <c r="E19" t="s">
         <v>51</v>
@@ -3446,14 +3350,8 @@
       <c r="A20" t="s">
         <v>106</v>
       </c>
-      <c r="B20" t="s">
-        <v>679</v>
-      </c>
       <c r="C20" t="s">
         <v>107</v>
-      </c>
-      <c r="D20" t="s">
-        <v>680</v>
       </c>
       <c r="E20" t="s">
         <v>19</v>
@@ -3478,14 +3376,8 @@
       <c r="A21" t="s">
         <v>111</v>
       </c>
-      <c r="B21" t="s">
-        <v>679</v>
-      </c>
       <c r="C21" t="s">
         <v>112</v>
-      </c>
-      <c r="D21" t="s">
-        <v>680</v>
       </c>
       <c r="E21" t="s">
         <v>27</v>
@@ -3510,14 +3402,8 @@
       <c r="A22" t="s">
         <v>118</v>
       </c>
-      <c r="B22" t="s">
-        <v>679</v>
-      </c>
       <c r="C22" t="s">
         <v>119</v>
-      </c>
-      <c r="D22" t="s">
-        <v>680</v>
       </c>
       <c r="E22" t="s">
         <v>35</v>
@@ -3542,14 +3428,8 @@
       <c r="A23" t="s">
         <v>122</v>
       </c>
-      <c r="B23" t="s">
-        <v>679</v>
-      </c>
       <c r="C23" t="s">
         <v>123</v>
-      </c>
-      <c r="D23" t="s">
-        <v>680</v>
       </c>
       <c r="E23" t="s">
         <v>43</v>
@@ -3574,14 +3454,8 @@
       <c r="A24" t="s">
         <v>128</v>
       </c>
-      <c r="B24" t="s">
-        <v>679</v>
-      </c>
       <c r="C24" t="s">
         <v>129</v>
-      </c>
-      <c r="D24" t="s">
-        <v>680</v>
       </c>
       <c r="E24" t="s">
         <v>51</v>
@@ -3606,14 +3480,8 @@
       <c r="A25" t="s">
         <v>134</v>
       </c>
-      <c r="B25" t="s">
-        <v>679</v>
-      </c>
       <c r="C25" t="s">
         <v>135</v>
-      </c>
-      <c r="D25" t="s">
-        <v>17</v>
       </c>
       <c r="E25" t="s">
         <v>19</v>
@@ -3638,14 +3506,8 @@
       <c r="A26" t="s">
         <v>140</v>
       </c>
-      <c r="B26" t="s">
-        <v>679</v>
-      </c>
       <c r="C26" t="s">
         <v>141</v>
-      </c>
-      <c r="D26" t="s">
-        <v>17</v>
       </c>
       <c r="E26" t="s">
         <v>27</v>
@@ -3670,14 +3532,8 @@
       <c r="A27" t="s">
         <v>144</v>
       </c>
-      <c r="B27" t="s">
-        <v>679</v>
-      </c>
       <c r="C27" t="s">
         <v>145</v>
-      </c>
-      <c r="D27" t="s">
-        <v>17</v>
       </c>
       <c r="E27" t="s">
         <v>35</v>
@@ -3702,14 +3558,8 @@
       <c r="A28" t="s">
         <v>151</v>
       </c>
-      <c r="B28" t="s">
-        <v>679</v>
-      </c>
       <c r="C28" t="s">
         <v>152</v>
-      </c>
-      <c r="D28" t="s">
-        <v>17</v>
       </c>
       <c r="E28" t="s">
         <v>43</v>
@@ -3734,9 +3584,6 @@
       <c r="A29" t="s">
         <v>158</v>
       </c>
-      <c r="B29" t="s">
-        <v>679</v>
-      </c>
       <c r="C29" t="s">
         <v>159</v>
       </c>
@@ -3766,9 +3613,6 @@
       <c r="A30" t="s">
         <v>165</v>
       </c>
-      <c r="B30" t="s">
-        <v>679</v>
-      </c>
       <c r="C30" t="s">
         <v>166</v>
       </c>
@@ -3798,9 +3642,6 @@
       <c r="A31" t="s">
         <v>170</v>
       </c>
-      <c r="B31" t="s">
-        <v>679</v>
-      </c>
       <c r="C31" t="s">
         <v>171</v>
       </c>
@@ -3830,9 +3671,6 @@
       <c r="A32" t="s">
         <v>177</v>
       </c>
-      <c r="B32" t="s">
-        <v>679</v>
-      </c>
       <c r="C32" t="s">
         <v>178</v>
       </c>
@@ -3862,9 +3700,6 @@
       <c r="A33" t="s">
         <v>180</v>
       </c>
-      <c r="B33" t="s">
-        <v>679</v>
-      </c>
       <c r="C33" t="s">
         <v>181</v>
       </c>
@@ -3894,9 +3729,6 @@
       <c r="A34" t="s">
         <v>186</v>
       </c>
-      <c r="B34" t="s">
-        <v>679</v>
-      </c>
       <c r="C34" t="s">
         <v>187</v>
       </c>
@@ -3926,9 +3758,6 @@
       <c r="A35" t="s">
         <v>191</v>
       </c>
-      <c r="B35" t="s">
-        <v>679</v>
-      </c>
       <c r="C35" t="s">
         <v>192</v>
       </c>
@@ -3958,9 +3787,6 @@
       <c r="A36" t="s">
         <v>198</v>
       </c>
-      <c r="B36" t="s">
-        <v>679</v>
-      </c>
       <c r="C36" t="s">
         <v>199</v>
       </c>
@@ -3990,9 +3816,6 @@
       <c r="A37" t="s">
         <v>205</v>
       </c>
-      <c r="B37" t="s">
-        <v>679</v>
-      </c>
       <c r="C37" t="s">
         <v>206</v>
       </c>
@@ -4022,14 +3845,8 @@
       <c r="A38" t="s">
         <v>212</v>
       </c>
-      <c r="B38" t="s">
-        <v>679</v>
-      </c>
       <c r="C38" t="s">
         <v>213</v>
-      </c>
-      <c r="D38" t="s">
-        <v>17</v>
       </c>
       <c r="E38" t="s">
         <v>43</v>
@@ -4054,14 +3871,8 @@
       <c r="A39" t="s">
         <v>215</v>
       </c>
-      <c r="B39" t="s">
-        <v>679</v>
-      </c>
       <c r="C39" t="s">
         <v>216</v>
-      </c>
-      <c r="D39" t="s">
-        <v>17</v>
       </c>
       <c r="E39" t="s">
         <v>51</v>
@@ -4086,14 +3897,8 @@
       <c r="A40" t="s">
         <v>218</v>
       </c>
-      <c r="B40" t="s">
-        <v>679</v>
-      </c>
       <c r="C40" t="s">
         <v>219</v>
-      </c>
-      <c r="D40" t="s">
-        <v>17</v>
       </c>
       <c r="E40" t="s">
         <v>19</v>
@@ -4118,14 +3923,8 @@
       <c r="A41" t="s">
         <v>223</v>
       </c>
-      <c r="B41" t="s">
-        <v>679</v>
-      </c>
       <c r="C41" t="s">
         <v>224</v>
-      </c>
-      <c r="D41" t="s">
-        <v>680</v>
       </c>
       <c r="E41" t="s">
         <v>27</v>
@@ -4150,14 +3949,8 @@
       <c r="A42" t="s">
         <v>230</v>
       </c>
-      <c r="B42" t="s">
-        <v>679</v>
-      </c>
       <c r="C42" t="s">
         <v>231</v>
-      </c>
-      <c r="D42" t="s">
-        <v>17</v>
       </c>
       <c r="E42" t="s">
         <v>35</v>
@@ -4182,14 +3975,8 @@
       <c r="A43" t="s">
         <v>235</v>
       </c>
-      <c r="B43" t="s">
-        <v>679</v>
-      </c>
       <c r="C43" t="s">
         <v>236</v>
-      </c>
-      <c r="D43" t="s">
-        <v>17</v>
       </c>
       <c r="E43" t="s">
         <v>43</v>
@@ -4214,14 +4001,8 @@
       <c r="A44" t="s">
         <v>241</v>
       </c>
-      <c r="B44" t="s">
-        <v>679</v>
-      </c>
       <c r="C44" t="s">
         <v>242</v>
-      </c>
-      <c r="D44" t="s">
-        <v>17</v>
       </c>
       <c r="E44" t="s">
         <v>51</v>
@@ -4246,14 +4027,8 @@
       <c r="A45" t="s">
         <v>248</v>
       </c>
-      <c r="B45" t="s">
-        <v>679</v>
-      </c>
       <c r="C45" t="s">
         <v>249</v>
-      </c>
-      <c r="D45" t="s">
-        <v>17</v>
       </c>
       <c r="E45" t="s">
         <v>19</v>
@@ -4278,14 +4053,8 @@
       <c r="A46" t="s">
         <v>255</v>
       </c>
-      <c r="B46" t="s">
-        <v>679</v>
-      </c>
       <c r="C46" t="s">
         <v>256</v>
-      </c>
-      <c r="D46" t="s">
-        <v>17</v>
       </c>
       <c r="E46" t="s">
         <v>27</v>
@@ -4310,14 +4079,8 @@
       <c r="A47" t="s">
         <v>262</v>
       </c>
-      <c r="B47" t="s">
-        <v>679</v>
-      </c>
       <c r="C47" t="s">
         <v>263</v>
-      </c>
-      <c r="D47" t="s">
-        <v>680</v>
       </c>
       <c r="E47" t="s">
         <v>35</v>
@@ -4342,14 +4105,8 @@
       <c r="A48" t="s">
         <v>269</v>
       </c>
-      <c r="B48" t="s">
-        <v>679</v>
-      </c>
       <c r="C48" t="s">
         <v>270</v>
-      </c>
-      <c r="D48" t="s">
-        <v>680</v>
       </c>
       <c r="E48" t="s">
         <v>43</v>
@@ -4374,14 +4131,8 @@
       <c r="A49" t="s">
         <v>272</v>
       </c>
-      <c r="B49" t="s">
-        <v>17</v>
-      </c>
       <c r="C49" t="s">
         <v>273</v>
-      </c>
-      <c r="D49" t="s">
-        <v>680</v>
       </c>
       <c r="E49" t="s">
         <v>51</v>
@@ -4406,14 +4157,8 @@
       <c r="A50" t="s">
         <v>279</v>
       </c>
-      <c r="B50" t="s">
-        <v>17</v>
-      </c>
       <c r="C50" t="s">
         <v>280</v>
-      </c>
-      <c r="D50" t="s">
-        <v>680</v>
       </c>
       <c r="E50" t="s">
         <v>19</v>
@@ -4438,14 +4183,8 @@
       <c r="A51" t="s">
         <v>286</v>
       </c>
-      <c r="B51" t="s">
-        <v>17</v>
-      </c>
       <c r="C51" t="s">
         <v>287</v>
-      </c>
-      <c r="D51" t="s">
-        <v>680</v>
       </c>
       <c r="E51" t="s">
         <v>27</v>
@@ -4470,14 +4209,8 @@
       <c r="A52" t="s">
         <v>293</v>
       </c>
-      <c r="B52" t="s">
-        <v>17</v>
-      </c>
       <c r="C52" t="s">
         <v>294</v>
-      </c>
-      <c r="D52" t="s">
-        <v>680</v>
       </c>
       <c r="E52" t="s">
         <v>35</v>
@@ -4502,14 +4235,8 @@
       <c r="A53" t="s">
         <v>300</v>
       </c>
-      <c r="B53" t="s">
-        <v>17</v>
-      </c>
       <c r="C53" t="s">
         <v>301</v>
-      </c>
-      <c r="D53" t="s">
-        <v>680</v>
       </c>
       <c r="E53" t="s">
         <v>43</v>
@@ -4534,14 +4261,8 @@
       <c r="A54" t="s">
         <v>307</v>
       </c>
-      <c r="B54" t="s">
-        <v>17</v>
-      </c>
       <c r="C54" t="s">
         <v>308</v>
-      </c>
-      <c r="D54" t="s">
-        <v>680</v>
       </c>
       <c r="E54" t="s">
         <v>51</v>
@@ -4566,14 +4287,8 @@
       <c r="A55" t="s">
         <v>312</v>
       </c>
-      <c r="B55" t="s">
-        <v>17</v>
-      </c>
       <c r="C55" t="s">
         <v>313</v>
-      </c>
-      <c r="D55" t="s">
-        <v>680</v>
       </c>
       <c r="E55" t="s">
         <v>19</v>
@@ -4598,14 +4313,8 @@
       <c r="A56" t="s">
         <v>319</v>
       </c>
-      <c r="B56" t="s">
-        <v>17</v>
-      </c>
       <c r="C56" t="s">
         <v>320</v>
-      </c>
-      <c r="D56" t="s">
-        <v>680</v>
       </c>
       <c r="E56" t="s">
         <v>27</v>
@@ -4636,9 +4345,6 @@
       <c r="C57" t="s">
         <v>327</v>
       </c>
-      <c r="D57" t="s">
-        <v>680</v>
-      </c>
       <c r="E57" t="s">
         <v>35</v>
       </c>
@@ -4668,9 +4374,6 @@
       <c r="C58" t="s">
         <v>334</v>
       </c>
-      <c r="D58" t="s">
-        <v>680</v>
-      </c>
       <c r="E58" t="s">
         <v>43</v>
       </c>
@@ -4700,9 +4403,6 @@
       <c r="C59" t="s">
         <v>341</v>
       </c>
-      <c r="D59" t="s">
-        <v>680</v>
-      </c>
       <c r="E59" t="s">
         <v>51</v>
       </c>
@@ -4732,9 +4432,6 @@
       <c r="C60" t="s">
         <v>348</v>
       </c>
-      <c r="D60" t="s">
-        <v>680</v>
-      </c>
       <c r="E60" t="s">
         <v>19</v>
       </c>
@@ -4764,9 +4461,6 @@
       <c r="C61" t="s">
         <v>354</v>
       </c>
-      <c r="D61" t="s">
-        <v>680</v>
-      </c>
       <c r="E61" t="s">
         <v>27</v>
       </c>
@@ -4796,9 +4490,6 @@
       <c r="C62" t="s">
         <v>359</v>
       </c>
-      <c r="D62" t="s">
-        <v>680</v>
-      </c>
       <c r="E62" t="s">
         <v>35</v>
       </c>
@@ -4828,9 +4519,6 @@
       <c r="C63" t="s">
         <v>361</v>
       </c>
-      <c r="D63" t="s">
-        <v>680</v>
-      </c>
       <c r="E63" t="s">
         <v>43</v>
       </c>
@@ -4860,9 +4548,6 @@
       <c r="C64" t="s">
         <v>363</v>
       </c>
-      <c r="D64" t="s">
-        <v>17</v>
-      </c>
       <c r="E64" t="s">
         <v>51</v>
       </c>
@@ -4892,9 +4577,6 @@
       <c r="C65" t="s">
         <v>366</v>
       </c>
-      <c r="D65" t="s">
-        <v>17</v>
-      </c>
       <c r="E65" t="s">
         <v>19</v>
       </c>
@@ -4924,9 +4606,6 @@
       <c r="C66" t="s">
         <v>373</v>
       </c>
-      <c r="D66" t="s">
-        <v>680</v>
-      </c>
       <c r="E66" t="s">
         <v>27</v>
       </c>
@@ -4956,9 +4635,6 @@
       <c r="C67" t="s">
         <v>380</v>
       </c>
-      <c r="D67" t="s">
-        <v>680</v>
-      </c>
       <c r="E67" t="s">
         <v>35</v>
       </c>
@@ -4988,9 +4664,6 @@
       <c r="C68" t="s">
         <v>385</v>
       </c>
-      <c r="D68" t="s">
-        <v>680</v>
-      </c>
       <c r="E68" t="s">
         <v>43</v>
       </c>
@@ -5017,9 +4690,6 @@
       <c r="C69" t="s">
         <v>388</v>
       </c>
-      <c r="D69" t="s">
-        <v>680</v>
-      </c>
       <c r="E69" t="s">
         <v>51</v>
       </c>
@@ -5049,9 +4719,6 @@
       <c r="C70" t="s">
         <v>395</v>
       </c>
-      <c r="D70" t="s">
-        <v>680</v>
-      </c>
       <c r="E70" t="s">
         <v>19</v>
       </c>
@@ -5081,9 +4748,6 @@
       <c r="C71" t="s">
         <v>402</v>
       </c>
-      <c r="D71" t="s">
-        <v>680</v>
-      </c>
       <c r="E71" t="s">
         <v>27</v>
       </c>
@@ -5113,9 +4777,6 @@
       <c r="C72" t="s">
         <v>409</v>
       </c>
-      <c r="D72" t="s">
-        <v>680</v>
-      </c>
       <c r="E72" t="s">
         <v>35</v>
       </c>
@@ -5145,9 +4806,6 @@
       <c r="C73" t="s">
         <v>416</v>
       </c>
-      <c r="D73" t="s">
-        <v>680</v>
-      </c>
       <c r="E73" t="s">
         <v>43</v>
       </c>
@@ -5177,9 +4835,6 @@
       <c r="C74" t="s">
         <v>422</v>
       </c>
-      <c r="D74" t="s">
-        <v>680</v>
-      </c>
       <c r="E74" t="s">
         <v>51</v>
       </c>
@@ -5209,9 +4864,6 @@
       <c r="C75" t="s">
         <v>429</v>
       </c>
-      <c r="D75" t="s">
-        <v>680</v>
-      </c>
       <c r="E75" t="s">
         <v>19</v>
       </c>
@@ -5241,9 +4893,6 @@
       <c r="C76" t="s">
         <v>434</v>
       </c>
-      <c r="D76" t="s">
-        <v>680</v>
-      </c>
       <c r="E76" t="s">
         <v>27</v>
       </c>
@@ -5273,9 +4922,6 @@
       <c r="C77" t="s">
         <v>441</v>
       </c>
-      <c r="D77" t="s">
-        <v>680</v>
-      </c>
       <c r="E77" t="s">
         <v>35</v>
       </c>
@@ -5305,9 +4951,6 @@
       <c r="C78" t="s">
         <v>444</v>
       </c>
-      <c r="D78" t="s">
-        <v>680</v>
-      </c>
       <c r="E78" t="s">
         <v>43</v>
       </c>
@@ -5337,9 +4980,6 @@
       <c r="C79" t="s">
         <v>451</v>
       </c>
-      <c r="D79" t="s">
-        <v>680</v>
-      </c>
       <c r="E79" t="s">
         <v>51</v>
       </c>
@@ -5369,9 +5009,6 @@
       <c r="C80" t="s">
         <v>458</v>
       </c>
-      <c r="D80" t="s">
-        <v>680</v>
-      </c>
       <c r="E80" t="s">
         <v>19</v>
       </c>
@@ -5401,9 +5038,6 @@
       <c r="C81" t="s">
         <v>465</v>
       </c>
-      <c r="D81" t="s">
-        <v>680</v>
-      </c>
       <c r="E81" t="s">
         <v>27</v>
       </c>
@@ -5433,9 +5067,6 @@
       <c r="C82" t="s">
         <v>470</v>
       </c>
-      <c r="D82" t="s">
-        <v>680</v>
-      </c>
       <c r="E82" t="s">
         <v>35</v>
       </c>
@@ -5465,9 +5096,6 @@
       <c r="C83" t="s">
         <v>474</v>
       </c>
-      <c r="D83" t="s">
-        <v>680</v>
-      </c>
       <c r="E83" t="s">
         <v>43</v>
       </c>
@@ -5497,9 +5125,6 @@
       <c r="C84" t="s">
         <v>481</v>
       </c>
-      <c r="D84" t="s">
-        <v>17</v>
-      </c>
       <c r="E84" t="s">
         <v>51</v>
       </c>
@@ -5529,9 +5154,6 @@
       <c r="C85" t="s">
         <v>485</v>
       </c>
-      <c r="D85" t="s">
-        <v>17</v>
-      </c>
       <c r="E85" t="s">
         <v>19</v>
       </c>
@@ -5561,9 +5183,6 @@
       <c r="C86" t="s">
         <v>492</v>
       </c>
-      <c r="D86" t="s">
-        <v>17</v>
-      </c>
       <c r="E86" t="s">
         <v>27</v>
       </c>
@@ -5593,9 +5212,6 @@
       <c r="C87" t="s">
         <v>499</v>
       </c>
-      <c r="D87" t="s">
-        <v>17</v>
-      </c>
       <c r="E87" t="s">
         <v>35</v>
       </c>
@@ -5625,9 +5241,6 @@
       <c r="C88" t="s">
         <v>506</v>
       </c>
-      <c r="D88" t="s">
-        <v>17</v>
-      </c>
       <c r="E88" t="s">
         <v>43</v>
       </c>
@@ -5657,9 +5270,6 @@
       <c r="C89" t="s">
         <v>513</v>
       </c>
-      <c r="D89" t="s">
-        <v>17</v>
-      </c>
       <c r="E89" t="s">
         <v>51</v>
       </c>
@@ -5689,9 +5299,6 @@
       <c r="C90" t="s">
         <v>520</v>
       </c>
-      <c r="D90" t="s">
-        <v>17</v>
-      </c>
       <c r="E90" t="s">
         <v>19</v>
       </c>
@@ -5721,9 +5328,6 @@
       <c r="C91" t="s">
         <v>526</v>
       </c>
-      <c r="D91" t="s">
-        <v>17</v>
-      </c>
       <c r="E91" t="s">
         <v>27</v>
       </c>
@@ -5753,9 +5357,6 @@
       <c r="C92" t="s">
         <v>533</v>
       </c>
-      <c r="D92" t="s">
-        <v>17</v>
-      </c>
       <c r="E92" t="s">
         <v>35</v>
       </c>
@@ -5785,9 +5386,6 @@
       <c r="C93" t="s">
         <v>537</v>
       </c>
-      <c r="D93" t="s">
-        <v>17</v>
-      </c>
       <c r="E93" t="s">
         <v>43</v>
       </c>
@@ -5817,9 +5415,6 @@
       <c r="C94" t="s">
         <v>543</v>
       </c>
-      <c r="D94" t="s">
-        <v>17</v>
-      </c>
       <c r="E94" t="s">
         <v>43</v>
       </c>
@@ -5846,9 +5441,6 @@
       <c r="C95" t="s">
         <v>549</v>
       </c>
-      <c r="D95" t="s">
-        <v>17</v>
-      </c>
       <c r="E95" t="s">
         <v>19</v>
       </c>
@@ -5878,9 +5470,6 @@
       <c r="C96" t="s">
         <v>556</v>
       </c>
-      <c r="D96" t="s">
-        <v>17</v>
-      </c>
       <c r="E96" t="s">
         <v>27</v>
       </c>
@@ -5910,9 +5499,6 @@
       <c r="C97" t="s">
         <v>563</v>
       </c>
-      <c r="D97" t="s">
-        <v>17</v>
-      </c>
       <c r="E97" t="s">
         <v>35</v>
       </c>
@@ -5942,9 +5528,6 @@
       <c r="C98" t="s">
         <v>570</v>
       </c>
-      <c r="D98" t="s">
-        <v>17</v>
-      </c>
       <c r="E98" t="s">
         <v>43</v>
       </c>
@@ -5974,9 +5557,6 @@
       <c r="C99" t="s">
         <v>577</v>
       </c>
-      <c r="D99" t="s">
-        <v>17</v>
-      </c>
       <c r="E99" t="s">
         <v>51</v>
       </c>
@@ -6006,9 +5586,6 @@
       <c r="C100" t="s">
         <v>584</v>
       </c>
-      <c r="D100" t="s">
-        <v>17</v>
-      </c>
       <c r="E100" t="s">
         <v>19</v>
       </c>
@@ -6038,9 +5615,6 @@
       <c r="C101" t="s">
         <v>591</v>
       </c>
-      <c r="D101" t="s">
-        <v>17</v>
-      </c>
       <c r="E101" t="s">
         <v>27</v>
       </c>
@@ -6070,9 +5644,6 @@
       <c r="C102" t="s">
         <v>598</v>
       </c>
-      <c r="D102" t="s">
-        <v>17</v>
-      </c>
       <c r="E102" t="s">
         <v>35</v>
       </c>
@@ -6102,9 +5673,6 @@
       <c r="C103" t="s">
         <v>605</v>
       </c>
-      <c r="D103" t="s">
-        <v>17</v>
-      </c>
       <c r="E103" t="s">
         <v>43</v>
       </c>
@@ -6134,9 +5702,6 @@
       <c r="C104" t="s">
         <v>610</v>
       </c>
-      <c r="D104" t="s">
-        <v>17</v>
-      </c>
       <c r="E104" t="s">
         <v>51</v>
       </c>
@@ -6166,9 +5731,6 @@
       <c r="C105" t="s">
         <v>617</v>
       </c>
-      <c r="D105" t="s">
-        <v>17</v>
-      </c>
       <c r="E105" t="s">
         <v>19</v>
       </c>
@@ -6198,9 +5760,6 @@
       <c r="C106" t="s">
         <v>624</v>
       </c>
-      <c r="D106" t="s">
-        <v>17</v>
-      </c>
       <c r="E106" t="s">
         <v>27</v>
       </c>
@@ -6230,9 +5789,6 @@
       <c r="C107" t="s">
         <v>630</v>
       </c>
-      <c r="D107" t="s">
-        <v>17</v>
-      </c>
       <c r="E107" t="s">
         <v>35</v>
       </c>
@@ -6262,9 +5818,6 @@
       <c r="C108" t="s">
         <v>637</v>
       </c>
-      <c r="D108" t="s">
-        <v>17</v>
-      </c>
       <c r="E108" t="s">
         <v>43</v>
       </c>
@@ -6294,9 +5847,6 @@
       <c r="C109" t="s">
         <v>640</v>
       </c>
-      <c r="D109" t="s">
-        <v>17</v>
-      </c>
       <c r="E109" t="s">
         <v>51</v>
       </c>
@@ -6326,9 +5876,6 @@
       <c r="C110" t="s">
         <v>647</v>
       </c>
-      <c r="D110" t="s">
-        <v>17</v>
-      </c>
       <c r="E110" t="s">
         <v>19</v>
       </c>
@@ -6358,9 +5905,6 @@
       <c r="C111" t="s">
         <v>654</v>
       </c>
-      <c r="D111" t="s">
-        <v>17</v>
-      </c>
       <c r="E111" t="s">
         <v>27</v>
       </c>
@@ -6389,9 +5933,6 @@
       </c>
       <c r="C112" t="s">
         <v>661</v>
-      </c>
-      <c r="D112" t="s">
-        <v>17</v>
       </c>
       <c r="E112" t="s">
         <v>35</v>

</xml_diff>